<commit_message>
process latest Use Group source data
</commit_message>
<xml_diff>
--- a/input/Use Group Chart - Complete Use List with NAICS.xlsx
+++ b/input/Use Group Chart - Complete Use List with NAICS.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m_carper\Documents\GitHub\edr-use-query-tool\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nyco365-my.sharepoint.com/personal/mcarper_planning_nyc_gov/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E21BE1-1486-46FA-A78C-B7461BB5E13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{70C64CDC-EABD-49D6-92C4-DEA61709AE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0AE4C16F-F448-46F1-BC50-77AA8FF29434}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CF69924-4D7B-49E6-ADFC-15C8E9BB2002}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CF69924-4D7B-49E6-ADFC-15C8E9BB2002}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$K$1:$K$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$1:$D$244</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6725" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6714" uniqueCount="526">
   <si>
     <t>Use Group</t>
   </si>
@@ -1809,13 +1809,13 @@
     <t>459210 News dealers; 459210 Newsstands (i.e., permanent); 459210 Magazine stands (i.e., permanent)</t>
   </si>
   <si>
+    <t>NAICS join not performed b/c laundry and dry cleaning not separated at NAICS index level</t>
+  </si>
+  <si>
+    <t>If court is indoors, falls into UG VI Services #Health and fitness establishments#</t>
+  </si>
+  <si>
     <t>Not an official Zoning Resolution use - added manually, follows rules of #Schools#. See Zoning Resolution glossary for details: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>NAICS index assigned for tool usability, relationship not officially defined in Zoning Resolution. See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>See ZR Glossary for #accessory# definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
   </si>
   <si>
     <r>
@@ -2209,35 +2209,93 @@
     </r>
   </si>
   <si>
-    <t>See ZR Glossary for #self-service storage facility# definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>See ZR Glossary for #public parking garage# and #public parking lot# definitions: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>If court is indoors, use falls into UG VI Services #Health and fitness establishments#</t>
-  </si>
-  <si>
-    <t>NAICS join not performed b/c laundry and dry cleaning not separable at NAICS index level</t>
-  </si>
-  <si>
-    <t>NAICS indices assigned for tool usability, relationship not officially defined in Zoning Resolution. See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>NAICS index assigned for tool usability, not specified in the Zoning Resolution</t>
-  </si>
-  <si>
-    <t>NAICS index assigned for tool usability, not specified in the Zoning Resolution; See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>NAICS indices assigned for tool usability, not specified in the Zoning Resolution; See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+    <t>See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>See ZR Glossary for use definition:</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> https://zr.planning.nyc.gov/article-i/chapter-2#12-10; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NAICS index assigned for tool usability, relationship not officially defined in Zoning Resolution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>See ZR Glossary for #public parking garage# and #public parking lot# definitions:</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>See ZR Glossary for #self-service storage facility# definition:</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2333,13 +2391,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2411,7 +2462,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2533,9 +2584,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3331,7 +3379,7 @@
       <c r="I5" s="37"/>
       <c r="J5" s="37"/>
       <c r="K5" s="37" t="s">
-        <v>524</v>
+        <v>503</v>
       </c>
       <c r="L5" s="26" t="s">
         <v>47</v>
@@ -5341,7 +5389,7 @@
       <c r="I25" s="37"/>
       <c r="J25" s="37"/>
       <c r="K25" s="37" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="L25" s="26" t="s">
         <v>42</v>
@@ -10861,9 +10909,7 @@
       <c r="H80" s="37"/>
       <c r="I80" s="37"/>
       <c r="J80" s="37"/>
-      <c r="K80" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K80" s="37"/>
       <c r="L80" s="30" t="s">
         <v>166</v>
       </c>
@@ -11944,7 +11990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:36" ht="60" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:36" ht="33" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>163</v>
       </c>
@@ -11970,8 +12016,8 @@
       <c r="J91" s="37" t="s">
         <v>459</v>
       </c>
-      <c r="K91" s="38" t="s">
-        <v>528</v>
+      <c r="K91" s="37" t="s">
+        <v>522</v>
       </c>
       <c r="L91" s="30" t="s">
         <v>166</v>
@@ -12176,9 +12222,7 @@
       <c r="H93" s="37"/>
       <c r="I93" s="37"/>
       <c r="J93" s="37"/>
-      <c r="K93" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K93" s="37"/>
       <c r="L93" s="30" t="s">
         <v>166</v>
       </c>
@@ -12885,9 +12929,7 @@
       <c r="H100" s="37"/>
       <c r="I100" s="43"/>
       <c r="J100" s="37"/>
-      <c r="K100" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K100" s="37"/>
       <c r="L100" s="30" t="s">
         <v>166</v>
       </c>
@@ -12990,9 +13032,7 @@
       <c r="H101" s="37"/>
       <c r="I101" s="43"/>
       <c r="J101" s="37"/>
-      <c r="K101" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K101" s="37"/>
       <c r="L101" s="30" t="s">
         <v>166</v>
       </c>
@@ -16929,9 +16969,7 @@
       <c r="H140" s="41"/>
       <c r="I140" s="42"/>
       <c r="J140" s="37"/>
-      <c r="K140" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K140" s="37"/>
       <c r="L140" s="27" t="s">
         <v>41</v>
       </c>
@@ -17034,9 +17072,7 @@
       <c r="H141" s="41"/>
       <c r="I141" s="42"/>
       <c r="J141" s="37"/>
-      <c r="K141" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K141" s="37"/>
       <c r="L141" s="27" t="s">
         <v>41</v>
       </c>
@@ -17242,9 +17278,7 @@
       <c r="J143" s="37" t="s">
         <v>455</v>
       </c>
-      <c r="K143" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K143" s="37"/>
       <c r="L143" s="27" t="s">
         <v>41</v>
       </c>
@@ -17349,8 +17383,8 @@
       </c>
       <c r="I144" s="37"/>
       <c r="J144" s="37"/>
-      <c r="K144" s="37" t="s">
-        <v>529</v>
+      <c r="K144" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L144" s="27" t="s">
         <v>41</v>
@@ -17457,9 +17491,7 @@
       <c r="J145" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="K145" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K145" s="37"/>
       <c r="L145" s="27" t="s">
         <v>41</v>
       </c>
@@ -17562,9 +17594,7 @@
       <c r="J146" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="K146" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K146" s="37"/>
       <c r="L146" s="27" t="s">
         <v>41</v>
       </c>
@@ -17667,9 +17697,7 @@
       <c r="H147" s="37"/>
       <c r="I147" s="37"/>
       <c r="J147" s="37"/>
-      <c r="K147" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K147" s="37"/>
       <c r="L147" s="27" t="s">
         <v>41</v>
       </c>
@@ -17771,7 +17799,7 @@
       <c r="I148" s="41"/>
       <c r="J148" s="41"/>
       <c r="K148" s="37" t="s">
-        <v>525</v>
+        <v>502</v>
       </c>
       <c r="L148" s="27" t="s">
         <v>41</v>
@@ -17874,7 +17902,7 @@
       <c r="I149" s="41"/>
       <c r="J149" s="41"/>
       <c r="K149" s="37" t="s">
-        <v>525</v>
+        <v>502</v>
       </c>
       <c r="L149" s="27" t="s">
         <v>41</v>
@@ -17978,9 +18006,7 @@
       <c r="H150" s="37"/>
       <c r="I150" s="37"/>
       <c r="J150" s="37"/>
-      <c r="K150" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K150" s="37"/>
       <c r="L150" s="27" t="s">
         <v>41</v>
       </c>
@@ -18489,8 +18515,8 @@
       <c r="J155" s="37" t="s">
         <v>462</v>
       </c>
-      <c r="K155" s="38" t="s">
-        <v>526</v>
+      <c r="K155" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L155" s="27" t="s">
         <v>41</v>
@@ -18594,8 +18620,8 @@
       <c r="H156" s="37"/>
       <c r="I156" s="37"/>
       <c r="J156" s="37"/>
-      <c r="K156" s="38" t="s">
-        <v>526</v>
+      <c r="K156" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L156" s="27" t="s">
         <v>41</v>
@@ -18673,7 +18699,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="157" spans="1:36" ht="60" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:36" ht="75" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>290</v>
       </c>
@@ -18697,8 +18723,8 @@
       </c>
       <c r="I157" s="37"/>
       <c r="J157" s="37"/>
-      <c r="K157" s="37" t="s">
-        <v>503</v>
+      <c r="K157" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L157" s="27" t="s">
         <v>41</v>
@@ -21000,7 +21026,7 @@
       <c r="I180" s="37"/>
       <c r="J180" s="37"/>
       <c r="K180" s="44" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="L180" s="27" t="s">
         <v>41</v>
@@ -22402,7 +22428,7 @@
       <c r="I194" s="37"/>
       <c r="J194" s="37"/>
       <c r="K194" s="44" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="L194" s="27" t="s">
         <v>41</v>
@@ -22604,7 +22630,7 @@
       <c r="I196" s="37"/>
       <c r="J196" s="37"/>
       <c r="K196" s="44" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="L196" s="27" t="s">
         <v>41</v>
@@ -27536,8 +27562,12 @@
     <hyperlink ref="K180" r:id="rId1" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{B49153F7-A902-45C7-B6E2-03D9CDE5FB83}"/>
     <hyperlink ref="K194" r:id="rId2" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{80268D6C-40C0-4DC9-B429-2CE028CF3FBC}"/>
     <hyperlink ref="K196" r:id="rId3" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{3604A234-D9D7-4312-B175-B52FC2B2235B}"/>
+    <hyperlink ref="K144" r:id="rId4" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{55814B34-C655-4F14-862B-551A5076E00E}"/>
+    <hyperlink ref="K155" r:id="rId5" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{8E21CFDE-3EDB-4494-A6DF-4DB265DCEEBA}"/>
+    <hyperlink ref="K156" r:id="rId6" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{1EAA61C2-1851-444D-ACB7-CC688FFC5E3C}"/>
+    <hyperlink ref="K157" r:id="rId7" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{2FD13ADB-E236-4104-8DF2-6A635000DE1B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
use note edits, expanded use term footnote
</commit_message>
<xml_diff>
--- a/input/Use Group Chart - Complete Use List with NAICS.xlsx
+++ b/input/Use Group Chart - Complete Use List with NAICS.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m_carper\Documents\GitHub\edr-use-query-tool\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nyco365-my.sharepoint.com/personal/mcarper_planning_nyc_gov/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E21BE1-1486-46FA-A78C-B7461BB5E13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{70C64CDC-EABD-49D6-92C4-DEA61709AE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0AE4C16F-F448-46F1-BC50-77AA8FF29434}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CF69924-4D7B-49E6-ADFC-15C8E9BB2002}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CF69924-4D7B-49E6-ADFC-15C8E9BB2002}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$K$1:$K$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$1:$D$244</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6725" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6714" uniqueCount="526">
   <si>
     <t>Use Group</t>
   </si>
@@ -1809,13 +1809,13 @@
     <t>459210 News dealers; 459210 Newsstands (i.e., permanent); 459210 Magazine stands (i.e., permanent)</t>
   </si>
   <si>
+    <t>NAICS join not performed b/c laundry and dry cleaning not separated at NAICS index level</t>
+  </si>
+  <si>
+    <t>If court is indoors, falls into UG VI Services #Health and fitness establishments#</t>
+  </si>
+  <si>
     <t>Not an official Zoning Resolution use - added manually, follows rules of #Schools#. See Zoning Resolution glossary for details: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>NAICS index assigned for tool usability, relationship not officially defined in Zoning Resolution. See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>See ZR Glossary for #accessory# definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
   </si>
   <si>
     <r>
@@ -2209,35 +2209,93 @@
     </r>
   </si>
   <si>
-    <t>See ZR Glossary for #self-service storage facility# definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>See ZR Glossary for #public parking garage# and #public parking lot# definitions: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>If court is indoors, use falls into UG VI Services #Health and fitness establishments#</t>
-  </si>
-  <si>
-    <t>NAICS join not performed b/c laundry and dry cleaning not separable at NAICS index level</t>
-  </si>
-  <si>
-    <t>NAICS indices assigned for tool usability, relationship not officially defined in Zoning Resolution. See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>NAICS index assigned for tool usability, not specified in the Zoning Resolution</t>
-  </si>
-  <si>
-    <t>NAICS index assigned for tool usability, not specified in the Zoning Resolution; See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>NAICS indices assigned for tool usability, not specified in the Zoning Resolution; See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+    <t>See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>See ZR Glossary for use definition:</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> https://zr.planning.nyc.gov/article-i/chapter-2#12-10; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NAICS index assigned for tool usability, relationship not officially defined in Zoning Resolution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>See ZR Glossary for #public parking garage# and #public parking lot# definitions:</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>See ZR Glossary for #self-service storage facility# definition:</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2333,13 +2391,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2411,7 +2462,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2533,9 +2584,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3331,7 +3379,7 @@
       <c r="I5" s="37"/>
       <c r="J5" s="37"/>
       <c r="K5" s="37" t="s">
-        <v>524</v>
+        <v>503</v>
       </c>
       <c r="L5" s="26" t="s">
         <v>47</v>
@@ -5341,7 +5389,7 @@
       <c r="I25" s="37"/>
       <c r="J25" s="37"/>
       <c r="K25" s="37" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="L25" s="26" t="s">
         <v>42</v>
@@ -10861,9 +10909,7 @@
       <c r="H80" s="37"/>
       <c r="I80" s="37"/>
       <c r="J80" s="37"/>
-      <c r="K80" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K80" s="37"/>
       <c r="L80" s="30" t="s">
         <v>166</v>
       </c>
@@ -11944,7 +11990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:36" ht="60" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:36" ht="33" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>163</v>
       </c>
@@ -11970,8 +12016,8 @@
       <c r="J91" s="37" t="s">
         <v>459</v>
       </c>
-      <c r="K91" s="38" t="s">
-        <v>528</v>
+      <c r="K91" s="37" t="s">
+        <v>522</v>
       </c>
       <c r="L91" s="30" t="s">
         <v>166</v>
@@ -12176,9 +12222,7 @@
       <c r="H93" s="37"/>
       <c r="I93" s="37"/>
       <c r="J93" s="37"/>
-      <c r="K93" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K93" s="37"/>
       <c r="L93" s="30" t="s">
         <v>166</v>
       </c>
@@ -12885,9 +12929,7 @@
       <c r="H100" s="37"/>
       <c r="I100" s="43"/>
       <c r="J100" s="37"/>
-      <c r="K100" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K100" s="37"/>
       <c r="L100" s="30" t="s">
         <v>166</v>
       </c>
@@ -12990,9 +13032,7 @@
       <c r="H101" s="37"/>
       <c r="I101" s="43"/>
       <c r="J101" s="37"/>
-      <c r="K101" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K101" s="37"/>
       <c r="L101" s="30" t="s">
         <v>166</v>
       </c>
@@ -16929,9 +16969,7 @@
       <c r="H140" s="41"/>
       <c r="I140" s="42"/>
       <c r="J140" s="37"/>
-      <c r="K140" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K140" s="37"/>
       <c r="L140" s="27" t="s">
         <v>41</v>
       </c>
@@ -17034,9 +17072,7 @@
       <c r="H141" s="41"/>
       <c r="I141" s="42"/>
       <c r="J141" s="37"/>
-      <c r="K141" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K141" s="37"/>
       <c r="L141" s="27" t="s">
         <v>41</v>
       </c>
@@ -17242,9 +17278,7 @@
       <c r="J143" s="37" t="s">
         <v>455</v>
       </c>
-      <c r="K143" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K143" s="37"/>
       <c r="L143" s="27" t="s">
         <v>41</v>
       </c>
@@ -17349,8 +17383,8 @@
       </c>
       <c r="I144" s="37"/>
       <c r="J144" s="37"/>
-      <c r="K144" s="37" t="s">
-        <v>529</v>
+      <c r="K144" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L144" s="27" t="s">
         <v>41</v>
@@ -17457,9 +17491,7 @@
       <c r="J145" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="K145" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K145" s="37"/>
       <c r="L145" s="27" t="s">
         <v>41</v>
       </c>
@@ -17562,9 +17594,7 @@
       <c r="J146" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="K146" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K146" s="37"/>
       <c r="L146" s="27" t="s">
         <v>41</v>
       </c>
@@ -17667,9 +17697,7 @@
       <c r="H147" s="37"/>
       <c r="I147" s="37"/>
       <c r="J147" s="37"/>
-      <c r="K147" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K147" s="37"/>
       <c r="L147" s="27" t="s">
         <v>41</v>
       </c>
@@ -17771,7 +17799,7 @@
       <c r="I148" s="41"/>
       <c r="J148" s="41"/>
       <c r="K148" s="37" t="s">
-        <v>525</v>
+        <v>502</v>
       </c>
       <c r="L148" s="27" t="s">
         <v>41</v>
@@ -17874,7 +17902,7 @@
       <c r="I149" s="41"/>
       <c r="J149" s="41"/>
       <c r="K149" s="37" t="s">
-        <v>525</v>
+        <v>502</v>
       </c>
       <c r="L149" s="27" t="s">
         <v>41</v>
@@ -17978,9 +18006,7 @@
       <c r="H150" s="37"/>
       <c r="I150" s="37"/>
       <c r="J150" s="37"/>
-      <c r="K150" s="45" t="s">
-        <v>527</v>
-      </c>
+      <c r="K150" s="37"/>
       <c r="L150" s="27" t="s">
         <v>41</v>
       </c>
@@ -18489,8 +18515,8 @@
       <c r="J155" s="37" t="s">
         <v>462</v>
       </c>
-      <c r="K155" s="38" t="s">
-        <v>526</v>
+      <c r="K155" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L155" s="27" t="s">
         <v>41</v>
@@ -18594,8 +18620,8 @@
       <c r="H156" s="37"/>
       <c r="I156" s="37"/>
       <c r="J156" s="37"/>
-      <c r="K156" s="38" t="s">
-        <v>526</v>
+      <c r="K156" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L156" s="27" t="s">
         <v>41</v>
@@ -18673,7 +18699,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="157" spans="1:36" ht="60" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:36" ht="75" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>290</v>
       </c>
@@ -18697,8 +18723,8 @@
       </c>
       <c r="I157" s="37"/>
       <c r="J157" s="37"/>
-      <c r="K157" s="37" t="s">
-        <v>503</v>
+      <c r="K157" s="44" t="s">
+        <v>523</v>
       </c>
       <c r="L157" s="27" t="s">
         <v>41</v>
@@ -21000,7 +21026,7 @@
       <c r="I180" s="37"/>
       <c r="J180" s="37"/>
       <c r="K180" s="44" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="L180" s="27" t="s">
         <v>41</v>
@@ -22402,7 +22428,7 @@
       <c r="I194" s="37"/>
       <c r="J194" s="37"/>
       <c r="K194" s="44" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="L194" s="27" t="s">
         <v>41</v>
@@ -22604,7 +22630,7 @@
       <c r="I196" s="37"/>
       <c r="J196" s="37"/>
       <c r="K196" s="44" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="L196" s="27" t="s">
         <v>41</v>
@@ -27536,8 +27562,12 @@
     <hyperlink ref="K180" r:id="rId1" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{B49153F7-A902-45C7-B6E2-03D9CDE5FB83}"/>
     <hyperlink ref="K194" r:id="rId2" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{80268D6C-40C0-4DC9-B429-2CE028CF3FBC}"/>
     <hyperlink ref="K196" r:id="rId3" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{3604A234-D9D7-4312-B175-B52FC2B2235B}"/>
+    <hyperlink ref="K144" r:id="rId4" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{55814B34-C655-4F14-862B-551A5076E00E}"/>
+    <hyperlink ref="K155" r:id="rId5" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{8E21CFDE-3EDB-4494-A6DF-4DB265DCEEBA}"/>
+    <hyperlink ref="K156" r:id="rId6" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{1EAA61C2-1851-444D-ACB7-CC688FFC5E3C}"/>
+    <hyperlink ref="K157" r:id="rId7" location="12-10" display="https://zr.planning.nyc.gov/article-i/chapter-2#12-10" xr:uid="{2FD13ADB-E236-4104-8DF2-6A635000DE1B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>